<commit_message>
update SVM partial results
</commit_message>
<xml_diff>
--- a/results/day_tractor/shallow/SVM/all_results_svm.xlsx
+++ b/results/day_tractor/shallow/SVM/all_results_svm.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK25"/>
+  <dimension ref="A1:AK26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3505,6 +3505,127 @@
       </c>
       <c r="AK25" t="n">
         <v>0.6588216601039006</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-06-24_16-18-41</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>42</v>
+      </c>
+      <c r="D26" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>72.15177748314311</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.2194704913043539</v>
+      </c>
+      <c r="H26" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>21</v>
+      </c>
+      <c r="L26" t="n">
+        <v>9937.740738236927</v>
+      </c>
+      <c r="M26" t="n">
+        <v>38560</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0.7593164016140518</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.8418188604857175</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.7593164016140518</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.7934024883141519</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0.8578670371872288</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0.6609506690632746</v>
+      </c>
+      <c r="T26" t="n">
+        <v>0.7213068956878915</v>
+      </c>
+      <c r="U26" t="n">
+        <v>0.6759295391854732</v>
+      </c>
+      <c r="V26" t="n">
+        <v>0.6905191633931416</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.6727409107248429</v>
+      </c>
+      <c r="X26" t="n">
+        <v>0.6905191633931416</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>0.6777294618529985</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>0.8134903577325802</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>0.5604227913919527</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>0.5647759703236018</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>0.5543855338085703</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>0.755649145541427</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>0.7480450312929088</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>0.755649145541427</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>0.7402123990925663</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>0.8648427774412154</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>0.6310729859957629</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>0.6439520156898589</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>0.6179322383062137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>